<commit_message>
build: add new posts
</commit_message>
<xml_diff>
--- a/docs/assets/files/asiabudget.xlsx
+++ b/docs/assets/files/asiabudget.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\William Vandergraaf\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\William Vandergraaf\Documents\GitHub Repos\daniela-and-will-travel.github.io\src\assets\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E8AA76-F44D-4451-A5C0-49349148DFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A14DB21-CC7F-4D2E-90C5-76F927428354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Budget" sheetId="1" r:id="rId1"/>
     <sheet name="Budget By Person" sheetId="2" r:id="rId2"/>
-    <sheet name="Matthew Tab" sheetId="4" state="hidden" r:id="rId3"/>
+    <sheet name="Intial Expenses" sheetId="5" r:id="rId3"/>
+    <sheet name="Matthew Tab" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="48">
   <si>
     <t>PLACE &amp; MONEY</t>
   </si>
@@ -171,14 +172,24 @@
   <si>
     <t xml:space="preserve">Person 2 Personal Budget: </t>
   </si>
+  <si>
+    <t>INITIAL EXPENSES</t>
+  </si>
+  <si>
+    <t>Who Paid?</t>
+  </si>
+  <si>
+    <t>Half</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$$]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="#,##0.00\ [$đ-42A]"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -366,7 +377,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -470,6 +481,16 @@
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -488,13 +509,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -507,24 +525,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -804,37 +808,37 @@
     <col min="7" max="7" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="57" t="s">
+      <c r="C1" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="54"/>
-      <c r="E1" s="57" t="s">
+      <c r="D1" s="58"/>
+      <c r="E1" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="54"/>
-      <c r="G1" s="57" t="s">
+      <c r="F1" s="58"/>
+      <c r="G1" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="54"/>
-      <c r="I1" s="57" t="s">
+      <c r="H1" s="58"/>
+      <c r="I1" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="54"/>
-      <c r="K1" s="57" t="s">
+      <c r="J1" s="58"/>
+      <c r="K1" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="54"/>
-      <c r="M1" s="57" t="s">
+      <c r="L1" s="58"/>
+      <c r="M1" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="58"/>
-      <c r="O1" s="57"/>
-      <c r="P1" s="54"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="58"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -849,10 +853,10 @@
       <c r="AB1" s="1"/>
     </row>
     <row r="2" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="52"/>
+      <c r="B2" s="56"/>
       <c r="C2" s="4"/>
       <c r="D2" s="5"/>
       <c r="E2" s="6"/>
@@ -880,7 +884,7 @@
       <c r="AA2" s="10"/>
       <c r="AB2" s="10"/>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>0</v>
       </c>
@@ -914,7 +918,7 @@
       <c r="AA3" s="15"/>
       <c r="AB3" s="15"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" s="17" t="e">
         <f>((N41/A40)*A3)-(SUM(C4:L4)+SUM(C5:L5))</f>
@@ -947,7 +951,7 @@
       <c r="AA4" s="15"/>
       <c r="AB4" s="15"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="20"/>
       <c r="B5" s="21"/>
       <c r="C5" s="4"/>
@@ -977,7 +981,7 @@
       <c r="AA5" s="10"/>
       <c r="AB5" s="10"/>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>0</v>
       </c>
@@ -1011,7 +1015,7 @@
       <c r="AA6" s="15"/>
       <c r="AB6" s="15"/>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
       <c r="B7" s="17" t="e">
         <f>((N41/A40)*A6)-(SUM(C7:N7)+L5+N8)</f>
@@ -1044,7 +1048,7 @@
       <c r="AA7" s="15"/>
       <c r="AB7" s="15"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A8" s="20"/>
       <c r="B8" s="21"/>
       <c r="C8" s="4"/>
@@ -1074,7 +1078,7 @@
       <c r="AA8" s="10"/>
       <c r="AB8" s="10"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>0</v>
       </c>
@@ -1108,7 +1112,7 @@
       <c r="AA9" s="15"/>
       <c r="AB9" s="15"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="17" t="e">
         <f>((N41/A40)*A9)-(SUM(C10:N10)+L11+N11)</f>
@@ -1141,7 +1145,7 @@
       <c r="AA10" s="15"/>
       <c r="AB10" s="15"/>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="20"/>
       <c r="B11" s="21"/>
       <c r="C11" s="10"/>
@@ -1171,7 +1175,7 @@
       <c r="AA11" s="10"/>
       <c r="AB11" s="10"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>0</v>
       </c>
@@ -1205,7 +1209,7 @@
       <c r="AA12" s="25"/>
       <c r="AB12" s="25"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="17" t="e">
         <f>((N41/A40)*A12)-(SUM(C13:N13)+L14+N14)</f>
@@ -1238,7 +1242,7 @@
       <c r="AA13" s="15"/>
       <c r="AB13" s="15"/>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A14" s="20"/>
       <c r="B14" s="21"/>
       <c r="C14" s="10"/>
@@ -1268,7 +1272,7 @@
       <c r="AA14" s="10"/>
       <c r="AB14" s="10"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>0</v>
       </c>
@@ -1302,7 +1306,7 @@
       <c r="AA15" s="25"/>
       <c r="AB15" s="25"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
       <c r="B16" s="17" t="e">
         <f>((N41/A40)*A15)-(SUM(C16:N16)+L17+N17)</f>
@@ -1335,7 +1339,7 @@
       <c r="AA16" s="15"/>
       <c r="AB16" s="15"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A17" s="20"/>
       <c r="B17" s="21"/>
       <c r="C17" s="10"/>
@@ -1365,7 +1369,7 @@
       <c r="AA17" s="10"/>
       <c r="AB17" s="10"/>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>0</v>
       </c>
@@ -1399,7 +1403,7 @@
       <c r="AA18" s="25"/>
       <c r="AB18" s="25"/>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="17" t="e">
         <f>((N41/A40)*A18)-(SUM(C19:N19)+L20+N20)</f>
@@ -1432,7 +1436,7 @@
       <c r="AA19" s="15"/>
       <c r="AB19" s="15"/>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A20" s="20"/>
       <c r="B20" s="21"/>
       <c r="C20" s="10"/>
@@ -1462,7 +1466,7 @@
       <c r="AA20" s="10"/>
       <c r="AB20" s="10"/>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>0</v>
       </c>
@@ -1496,7 +1500,7 @@
       <c r="AA21" s="25"/>
       <c r="AB21" s="25"/>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="17" t="e">
         <f>((N41/A40)*A21)-(SUM(C22:N22)+L23+N23)</f>
@@ -1529,7 +1533,7 @@
       <c r="AA22" s="15"/>
       <c r="AB22" s="15"/>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
       <c r="B23" s="21"/>
       <c r="C23" s="10"/>
@@ -1559,7 +1563,7 @@
       <c r="AA23" s="10"/>
       <c r="AB23" s="10"/>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>0</v>
       </c>
@@ -1593,7 +1597,7 @@
       <c r="AA24" s="25"/>
       <c r="AB24" s="25"/>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="17" t="e">
         <f>((N41/A40)*A24)-(SUM(C25:N25)+L26+N26)</f>
@@ -1626,7 +1630,7 @@
       <c r="AA25" s="15"/>
       <c r="AB25" s="15"/>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A26" s="20"/>
       <c r="B26" s="21"/>
       <c r="C26" s="10"/>
@@ -1656,7 +1660,7 @@
       <c r="AA26" s="10"/>
       <c r="AB26" s="10"/>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>0</v>
       </c>
@@ -1690,7 +1694,7 @@
       <c r="AA27" s="25"/>
       <c r="AB27" s="25"/>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="17" t="e">
         <f>((N41/A40)*A27)-(SUM(C28:N28)+L29+N29)</f>
@@ -2045,10 +2049,10 @@
       <c r="AB38" s="10"/>
     </row>
     <row r="39" spans="1:28" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="53" t="s">
+      <c r="A39" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="54"/>
+      <c r="B39" s="58"/>
       <c r="C39" s="4"/>
       <c r="D39" s="5"/>
       <c r="E39" s="23"/>
@@ -2144,19 +2148,19 @@
     <row r="41" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A41" s="33"/>
       <c r="B41" s="34"/>
-      <c r="C41" s="55" t="s">
+      <c r="C41" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="D41" s="54"/>
-      <c r="E41" s="54"/>
-      <c r="F41" s="54"/>
-      <c r="G41" s="54"/>
-      <c r="H41" s="54"/>
-      <c r="I41" s="54"/>
-      <c r="J41" s="54"/>
-      <c r="K41" s="54"/>
-      <c r="L41" s="54"/>
-      <c r="M41" s="54"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="58"/>
+      <c r="G41" s="58"/>
+      <c r="H41" s="58"/>
+      <c r="I41" s="58"/>
+      <c r="J41" s="58"/>
+      <c r="K41" s="58"/>
+      <c r="L41" s="58"/>
+      <c r="M41" s="58"/>
       <c r="N41" s="35"/>
       <c r="O41" s="15"/>
       <c r="P41" s="15"/>
@@ -2176,24 +2180,24 @@
     <row r="42" spans="1:28" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
       <c r="B42" s="36"/>
-      <c r="C42" s="56" t="s">
+      <c r="C42" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="D42" s="54"/>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="54"/>
-      <c r="H42" s="54"/>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54"/>
+      <c r="D42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="58"/>
+      <c r="G42" s="58"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
+      <c r="J42" s="58"/>
       <c r="K42" s="37">
         <f>D40+F40+H40+J40+L40+N40</f>
         <v>0</v>
       </c>
-      <c r="L42" s="56" t="s">
+      <c r="L42" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="M42" s="54"/>
+      <c r="M42" s="58"/>
       <c r="N42" s="38">
         <f>SUM(N41-K42)</f>
         <v>0</v>
@@ -30910,26 +30914,26 @@
     <col min="16" max="16" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+    <row r="1" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="63" t="s">
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="65"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="68"/>
       <c r="N1" s="25"/>
       <c r="O1" s="25"/>
       <c r="P1" s="25"/>
@@ -30945,32 +30949,32 @@
       <c r="Z1" s="25"/>
       <c r="AA1" s="25"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A2" s="54"/>
-      <c r="B2" s="59" t="s">
+    <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="58"/>
+      <c r="B2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="59" t="s">
+      <c r="C2" s="58"/>
+      <c r="D2" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="54"/>
-      <c r="F2" s="59" t="s">
+      <c r="E2" s="58"/>
+      <c r="F2" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="58"/>
-      <c r="H2" s="59" t="s">
+      <c r="G2" s="62"/>
+      <c r="H2" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="54"/>
-      <c r="J2" s="59" t="s">
+      <c r="I2" s="58"/>
+      <c r="J2" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="54"/>
-      <c r="L2" s="59" t="s">
+      <c r="K2" s="58"/>
+      <c r="L2" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="58"/>
+      <c r="M2" s="62"/>
       <c r="N2" s="25"/>
       <c r="O2" s="25"/>
       <c r="P2" s="25"/>
@@ -30986,8 +30990,8 @@
       <c r="Z2" s="25"/>
       <c r="AA2" s="25"/>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A3" s="54"/>
+    <row r="3" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A3" s="58"/>
       <c r="B3" s="36"/>
       <c r="C3" s="40"/>
       <c r="D3" s="36"/>
@@ -31019,838 +31023,838 @@
       <c r="A4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="67">
+      <c r="B4" s="36">
         <f>(Budget!D2)/2</f>
         <v>0</v>
       </c>
-      <c r="C4" s="68">
+      <c r="C4" s="40">
         <f>B4</f>
         <v>0</v>
       </c>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="67"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="67"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="69"/>
-      <c r="O4" s="69"/>
-      <c r="P4" s="69"/>
-      <c r="Q4" s="69"/>
-      <c r="R4" s="69"/>
-      <c r="S4" s="69"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="69"/>
-      <c r="V4" s="69"/>
-      <c r="W4" s="69"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="16"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="16"/>
+      <c r="W4" s="16"/>
       <c r="X4" s="16"/>
       <c r="Y4" s="16"/>
       <c r="Z4" s="16"/>
       <c r="AA4" s="16"/>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="67">
+      <c r="B5" s="36">
         <f>(Budget!D5)/2</f>
         <v>0</v>
       </c>
-      <c r="C5" s="68">
+      <c r="C5" s="40">
         <f>(Budget!D4)/2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="67">
+      <c r="D5" s="36">
         <f>(Budget!F5)/2</f>
         <v>0</v>
       </c>
-      <c r="E5" s="68">
+      <c r="E5" s="40">
         <f>(Budget!F4)/2</f>
         <v>0</v>
       </c>
-      <c r="F5" s="67">
+      <c r="F5" s="36">
         <f>(Budget!H5)/2</f>
         <v>0</v>
       </c>
-      <c r="G5" s="68">
+      <c r="G5" s="40">
         <f>(Budget!H4)/2</f>
         <v>0</v>
       </c>
-      <c r="H5" s="67">
+      <c r="H5" s="36">
         <f>(Budget!J5)/2</f>
         <v>0</v>
       </c>
-      <c r="I5" s="68">
+      <c r="I5" s="40">
         <f>(Budget!J4)/2</f>
         <v>0</v>
       </c>
-      <c r="J5" s="68">
+      <c r="J5" s="40">
         <f>(Budget!L5)/2</f>
         <v>0</v>
       </c>
-      <c r="K5" s="68">
+      <c r="K5" s="40">
         <f>(Budget!L4)/2</f>
         <v>0</v>
       </c>
-      <c r="L5" s="67">
+      <c r="L5" s="36">
         <f>(Budget!N5)/2</f>
         <v>0</v>
       </c>
-      <c r="M5" s="68">
+      <c r="M5" s="40">
         <f>(Budget!N4)/2</f>
         <v>0</v>
       </c>
-      <c r="N5" s="70"/>
-      <c r="O5" s="70"/>
-      <c r="P5" s="71"/>
-      <c r="Q5" s="71"/>
-      <c r="R5" s="71"/>
-      <c r="S5" s="71"/>
-      <c r="T5" s="71"/>
-      <c r="U5" s="71"/>
-      <c r="V5" s="71"/>
-      <c r="W5" s="71"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15"/>
+      <c r="V5" s="15"/>
+      <c r="W5" s="15"/>
       <c r="X5" s="15"/>
       <c r="Y5" s="15"/>
       <c r="Z5" s="15"/>
       <c r="AA5" s="15"/>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="67">
+      <c r="B6" s="36">
         <f>(Budget!D8)/2</f>
         <v>0</v>
       </c>
-      <c r="C6" s="68">
+      <c r="C6" s="40">
         <f>(Budget!D7)/2</f>
         <v>0</v>
       </c>
-      <c r="D6" s="67">
+      <c r="D6" s="36">
         <f>(Budget!F8)/2</f>
         <v>0</v>
       </c>
-      <c r="E6" s="68">
+      <c r="E6" s="40">
         <f>(Budget!F7)/2</f>
         <v>0</v>
       </c>
-      <c r="F6" s="67">
+      <c r="F6" s="36">
         <f>(Budget!H8)/2</f>
         <v>0</v>
       </c>
-      <c r="G6" s="68">
+      <c r="G6" s="40">
         <f>(Budget!H7)/2</f>
         <v>0</v>
       </c>
-      <c r="H6" s="67">
+      <c r="H6" s="36">
         <f>(Budget!J8)/2</f>
         <v>0</v>
       </c>
-      <c r="I6" s="68">
+      <c r="I6" s="40">
         <f>(Budget!J7)/2</f>
         <v>0</v>
       </c>
-      <c r="J6" s="67">
+      <c r="J6" s="36">
         <f>(Budget!L5)/2</f>
         <v>0</v>
       </c>
-      <c r="K6" s="68">
+      <c r="K6" s="40">
         <f>(Budget!L7)/2</f>
         <v>0</v>
       </c>
-      <c r="L6" s="67">
+      <c r="L6" s="36">
         <f>(Budget!N8)/2</f>
         <v>0</v>
       </c>
-      <c r="M6" s="68">
+      <c r="M6" s="40">
         <f>(Budget!N7)/2</f>
         <v>0</v>
       </c>
-      <c r="N6" s="70"/>
-      <c r="O6" s="70"/>
-      <c r="P6" s="70"/>
-      <c r="Q6" s="71"/>
-      <c r="R6" s="71"/>
-      <c r="S6" s="71"/>
-      <c r="T6" s="71"/>
-      <c r="U6" s="71"/>
-      <c r="V6" s="71"/>
-      <c r="W6" s="71"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="15"/>
+      <c r="U6" s="15"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="15"/>
       <c r="X6" s="15"/>
       <c r="Y6" s="15"/>
       <c r="Z6" s="15"/>
       <c r="AA6" s="15"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="67">
+      <c r="B7" s="36">
         <f>(Budget!D11)/2</f>
         <v>0</v>
       </c>
-      <c r="C7" s="68">
+      <c r="C7" s="40">
         <f>(Budget!D10)/2</f>
         <v>0</v>
       </c>
-      <c r="D7" s="67">
+      <c r="D7" s="36">
         <f>(Budget!F11)/2</f>
         <v>0</v>
       </c>
-      <c r="E7" s="68">
+      <c r="E7" s="40">
         <f>(Budget!F10)/2</f>
         <v>0</v>
       </c>
-      <c r="F7" s="67">
+      <c r="F7" s="36">
         <f>(Budget!H11)/2</f>
         <v>0</v>
       </c>
-      <c r="G7" s="68">
+      <c r="G7" s="40">
         <f>(Budget!H10)/2</f>
         <v>0</v>
       </c>
-      <c r="H7" s="67">
+      <c r="H7" s="36">
         <f>(Budget!J11)/2</f>
         <v>0</v>
       </c>
-      <c r="I7" s="68">
+      <c r="I7" s="40">
         <f>(Budget!J10)/2</f>
         <v>0</v>
       </c>
-      <c r="J7" s="67">
+      <c r="J7" s="36">
         <f>(Budget!L11)/2</f>
         <v>0</v>
       </c>
-      <c r="K7" s="68">
+      <c r="K7" s="40">
         <f>(Budget!L10)/2</f>
         <v>0</v>
       </c>
-      <c r="L7" s="67">
+      <c r="L7" s="36">
         <f>(Budget!N11)/2</f>
         <v>0</v>
       </c>
-      <c r="M7" s="68">
+      <c r="M7" s="40">
         <f>(Budget!N10)/2</f>
         <v>0</v>
       </c>
-      <c r="N7" s="70"/>
-      <c r="O7" s="70"/>
-      <c r="P7" s="70"/>
-      <c r="Q7" s="71"/>
-      <c r="R7" s="71"/>
-      <c r="S7" s="71"/>
-      <c r="T7" s="71"/>
-      <c r="U7" s="71"/>
-      <c r="V7" s="71"/>
-      <c r="W7" s="71"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="15"/>
+      <c r="U7" s="15"/>
+      <c r="V7" s="15"/>
+      <c r="W7" s="15"/>
       <c r="X7" s="15"/>
       <c r="Y7" s="15"/>
       <c r="Z7" s="15"/>
       <c r="AA7" s="15"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="67">
+      <c r="B8" s="36">
         <f>(Budget!D14)/2</f>
         <v>0</v>
       </c>
-      <c r="C8" s="68">
+      <c r="C8" s="40">
         <f>(Budget!D13)/2</f>
         <v>0</v>
       </c>
-      <c r="D8" s="67">
+      <c r="D8" s="36">
         <f>(Budget!F14)/2</f>
         <v>0</v>
       </c>
-      <c r="E8" s="68">
+      <c r="E8" s="40">
         <f>(Budget!F13)/2</f>
         <v>0</v>
       </c>
-      <c r="F8" s="67">
+      <c r="F8" s="36">
         <f>(Budget!H14)/2</f>
         <v>0</v>
       </c>
-      <c r="G8" s="68">
+      <c r="G8" s="40">
         <f>(Budget!H13)/2</f>
         <v>0</v>
       </c>
-      <c r="H8" s="67">
+      <c r="H8" s="36">
         <f>(Budget!J14)/2</f>
         <v>0</v>
       </c>
-      <c r="I8" s="68">
+      <c r="I8" s="40">
         <f>(Budget!J13)/2</f>
         <v>0</v>
       </c>
-      <c r="J8" s="67">
+      <c r="J8" s="36">
         <f>(Budget!L14)/2</f>
         <v>0</v>
       </c>
-      <c r="K8" s="68">
+      <c r="K8" s="40">
         <f>(Budget!L13)/2</f>
         <v>0</v>
       </c>
-      <c r="L8" s="67">
+      <c r="L8" s="36">
         <f>(Budget!N14)/2</f>
         <v>0</v>
       </c>
-      <c r="M8" s="68">
+      <c r="M8" s="40">
         <f>(Budget!N13)/2</f>
         <v>0</v>
       </c>
-      <c r="N8" s="70"/>
-      <c r="O8" s="70"/>
-      <c r="P8" s="70"/>
-      <c r="Q8" s="71"/>
-      <c r="R8" s="71"/>
-      <c r="S8" s="71"/>
-      <c r="T8" s="71"/>
-      <c r="U8" s="71"/>
-      <c r="V8" s="71"/>
-      <c r="W8" s="71"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="15"/>
+      <c r="S8" s="15"/>
+      <c r="T8" s="15"/>
+      <c r="U8" s="15"/>
+      <c r="V8" s="15"/>
+      <c r="W8" s="15"/>
       <c r="X8" s="15"/>
       <c r="Y8" s="15"/>
       <c r="Z8" s="15"/>
       <c r="AA8" s="15"/>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="67">
+      <c r="B9" s="36">
         <f>(Budget!D17)/2</f>
         <v>0</v>
       </c>
-      <c r="C9" s="68">
+      <c r="C9" s="40">
         <f>(Budget!D16)/2</f>
         <v>0</v>
       </c>
-      <c r="D9" s="67">
+      <c r="D9" s="36">
         <f>(Budget!F17)/2</f>
         <v>0</v>
       </c>
-      <c r="E9" s="68">
+      <c r="E9" s="40">
         <f>(Budget!F16)/2</f>
         <v>0</v>
       </c>
-      <c r="F9" s="67">
+      <c r="F9" s="36">
         <f>(Budget!H17)/2</f>
         <v>0</v>
       </c>
-      <c r="G9" s="68">
+      <c r="G9" s="40">
         <f>(Budget!H16)/2</f>
         <v>0</v>
       </c>
-      <c r="H9" s="67">
+      <c r="H9" s="36">
         <f>(Budget!J17)/2</f>
         <v>0</v>
       </c>
-      <c r="I9" s="68">
+      <c r="I9" s="40">
         <f>(Budget!J16)/2</f>
         <v>0</v>
       </c>
-      <c r="J9" s="67">
+      <c r="J9" s="36">
         <f>(Budget!L17)/2</f>
         <v>0</v>
       </c>
-      <c r="K9" s="68">
+      <c r="K9" s="40">
         <f>(Budget!L16)/2</f>
         <v>0</v>
       </c>
-      <c r="L9" s="67">
+      <c r="L9" s="36">
         <f>(Budget!N17)/2</f>
         <v>0</v>
       </c>
-      <c r="M9" s="68">
+      <c r="M9" s="40">
         <f>(Budget!N16)/2</f>
         <v>0</v>
       </c>
-      <c r="N9" s="70"/>
-      <c r="O9" s="70"/>
-      <c r="P9" s="70"/>
-      <c r="Q9" s="71"/>
-      <c r="R9" s="71"/>
-      <c r="S9" s="71"/>
-      <c r="T9" s="71"/>
-      <c r="U9" s="71"/>
-      <c r="V9" s="71"/>
-      <c r="W9" s="71"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
+      <c r="T9" s="15"/>
+      <c r="U9" s="15"/>
+      <c r="V9" s="15"/>
+      <c r="W9" s="15"/>
       <c r="X9" s="15"/>
       <c r="Y9" s="15"/>
       <c r="Z9" s="15"/>
       <c r="AA9" s="15"/>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="67">
+      <c r="B10" s="36">
         <f>(Budget!D20)/2</f>
         <v>0</v>
       </c>
-      <c r="C10" s="68">
+      <c r="C10" s="40">
         <f>(Budget!D19)/2</f>
         <v>0</v>
       </c>
-      <c r="D10" s="67">
+      <c r="D10" s="36">
         <f>(Budget!F20)/2</f>
         <v>0</v>
       </c>
-      <c r="E10" s="68">
+      <c r="E10" s="40">
         <f>(Budget!F19)/2</f>
         <v>0</v>
       </c>
-      <c r="F10" s="67">
+      <c r="F10" s="36">
         <f>(Budget!H20)/2</f>
         <v>0</v>
       </c>
-      <c r="G10" s="68">
+      <c r="G10" s="40">
         <f>(Budget!H19)/2</f>
         <v>0</v>
       </c>
-      <c r="H10" s="67">
+      <c r="H10" s="36">
         <f>(Budget!J20)/2</f>
         <v>0</v>
       </c>
-      <c r="I10" s="68">
+      <c r="I10" s="40">
         <f>(Budget!J19)/2</f>
         <v>0</v>
       </c>
-      <c r="J10" s="67">
+      <c r="J10" s="36">
         <f>(Budget!L20)/2</f>
         <v>0</v>
       </c>
-      <c r="K10" s="68">
+      <c r="K10" s="40">
         <f>(Budget!L19)/2</f>
         <v>0</v>
       </c>
-      <c r="L10" s="67">
+      <c r="L10" s="36">
         <f>(Budget!N20)/2</f>
         <v>0</v>
       </c>
-      <c r="M10" s="68">
+      <c r="M10" s="40">
         <f>(Budget!N19)/2</f>
         <v>0</v>
       </c>
-      <c r="N10" s="70"/>
-      <c r="O10" s="70"/>
-      <c r="P10" s="70"/>
-      <c r="Q10" s="71"/>
-      <c r="R10" s="71"/>
-      <c r="S10" s="71"/>
-      <c r="T10" s="71"/>
-      <c r="U10" s="71"/>
-      <c r="V10" s="71"/>
-      <c r="W10" s="71"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
+      <c r="T10" s="15"/>
+      <c r="U10" s="15"/>
+      <c r="V10" s="15"/>
+      <c r="W10" s="15"/>
       <c r="X10" s="15"/>
       <c r="Y10" s="15"/>
       <c r="Z10" s="15"/>
       <c r="AA10" s="15"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="67">
+      <c r="B11" s="36">
         <f>(Budget!D23)/2</f>
         <v>0</v>
       </c>
-      <c r="C11" s="68">
+      <c r="C11" s="40">
         <f>(Budget!D22)/2</f>
         <v>0</v>
       </c>
-      <c r="D11" s="67">
+      <c r="D11" s="36">
         <f>(Budget!F23)/2</f>
         <v>0</v>
       </c>
-      <c r="E11" s="68">
+      <c r="E11" s="40">
         <f>(Budget!F22)/2</f>
         <v>0</v>
       </c>
-      <c r="F11" s="67">
+      <c r="F11" s="36">
         <f>(Budget!H23)/2</f>
         <v>0</v>
       </c>
-      <c r="G11" s="68">
+      <c r="G11" s="40">
         <f>(Budget!H22)/2</f>
         <v>0</v>
       </c>
-      <c r="H11" s="67">
+      <c r="H11" s="36">
         <f>(Budget!J23)/2</f>
         <v>0</v>
       </c>
-      <c r="I11" s="68">
+      <c r="I11" s="40">
         <f>(Budget!J22)/2</f>
         <v>0</v>
       </c>
-      <c r="J11" s="67">
+      <c r="J11" s="36">
         <f>(Budget!L23)/2</f>
         <v>0</v>
       </c>
-      <c r="K11" s="68">
+      <c r="K11" s="40">
         <f>(Budget!L22)/2</f>
         <v>0</v>
       </c>
-      <c r="L11" s="67">
+      <c r="L11" s="36">
         <f>(Budget!N23)/2</f>
         <v>0</v>
       </c>
-      <c r="M11" s="68">
+      <c r="M11" s="40">
         <f>(Budget!N22)/2</f>
         <v>0</v>
       </c>
-      <c r="N11" s="70"/>
-      <c r="O11" s="70"/>
-      <c r="P11" s="70"/>
-      <c r="Q11" s="71"/>
-      <c r="R11" s="71"/>
-      <c r="S11" s="71"/>
-      <c r="T11" s="71"/>
-      <c r="U11" s="71"/>
-      <c r="V11" s="71"/>
-      <c r="W11" s="71"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="15"/>
+      <c r="R11" s="15"/>
+      <c r="S11" s="15"/>
+      <c r="T11" s="15"/>
+      <c r="U11" s="15"/>
+      <c r="V11" s="15"/>
+      <c r="W11" s="15"/>
       <c r="X11" s="15"/>
       <c r="Y11" s="15"/>
       <c r="Z11" s="15"/>
       <c r="AA11" s="15"/>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="67">
+      <c r="B12" s="36">
         <f>(Budget!D26)/2</f>
         <v>0</v>
       </c>
-      <c r="C12" s="68">
+      <c r="C12" s="40">
         <f>(Budget!D25)/2</f>
         <v>0</v>
       </c>
-      <c r="D12" s="67">
+      <c r="D12" s="36">
         <f>(Budget!F26)/2</f>
         <v>0</v>
       </c>
-      <c r="E12" s="68">
+      <c r="E12" s="40">
         <f>(Budget!F25)/2</f>
         <v>0</v>
       </c>
-      <c r="F12" s="67">
+      <c r="F12" s="36">
         <f>(Budget!H26)/2</f>
         <v>0</v>
       </c>
-      <c r="G12" s="68">
+      <c r="G12" s="40">
         <f>(Budget!H25)/2</f>
         <v>0</v>
       </c>
-      <c r="H12" s="67">
+      <c r="H12" s="36">
         <f>(Budget!J26)/2</f>
         <v>0</v>
       </c>
-      <c r="I12" s="68">
+      <c r="I12" s="40">
         <f>(Budget!J25)/2</f>
         <v>0</v>
       </c>
-      <c r="J12" s="67">
+      <c r="J12" s="36">
         <f>(Budget!L26)/2</f>
         <v>0</v>
       </c>
-      <c r="K12" s="68">
+      <c r="K12" s="40">
         <f>(Budget!L25)/2</f>
         <v>0</v>
       </c>
-      <c r="L12" s="67">
+      <c r="L12" s="36">
         <f>(Budget!N26)/2</f>
         <v>0</v>
       </c>
-      <c r="M12" s="68">
+      <c r="M12" s="40">
         <f>(Budget!N25)/2</f>
         <v>0</v>
       </c>
-      <c r="N12" s="70"/>
-      <c r="O12" s="70"/>
-      <c r="P12" s="70"/>
-      <c r="Q12" s="71"/>
-      <c r="R12" s="71"/>
-      <c r="S12" s="71"/>
-      <c r="T12" s="71"/>
-      <c r="U12" s="71"/>
-      <c r="V12" s="71"/>
-      <c r="W12" s="71"/>
+      <c r="N12" s="14"/>
+      <c r="O12" s="14"/>
+      <c r="P12" s="14"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="15"/>
+      <c r="U12" s="15"/>
+      <c r="V12" s="15"/>
+      <c r="W12" s="15"/>
       <c r="X12" s="15"/>
       <c r="Y12" s="15"/>
       <c r="Z12" s="15"/>
       <c r="AA12" s="15"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="67">
+      <c r="B13" s="36">
         <f>(Budget!D29)/2</f>
         <v>0</v>
       </c>
-      <c r="C13" s="68">
+      <c r="C13" s="40">
         <f>(Budget!D28)/2</f>
         <v>0</v>
       </c>
-      <c r="D13" s="67">
+      <c r="D13" s="36">
         <f>(Budget!F29)/2</f>
         <v>0</v>
       </c>
-      <c r="E13" s="68">
+      <c r="E13" s="40">
         <f>(Budget!F28)/2</f>
         <v>0</v>
       </c>
-      <c r="F13" s="67">
+      <c r="F13" s="36">
         <f>(Budget!H29)/2</f>
         <v>0</v>
       </c>
-      <c r="G13" s="68">
+      <c r="G13" s="40">
         <f>(Budget!H28)/2</f>
         <v>0</v>
       </c>
-      <c r="H13" s="67">
+      <c r="H13" s="36">
         <f>(Budget!J29)/2</f>
         <v>0</v>
       </c>
-      <c r="I13" s="68">
+      <c r="I13" s="40">
         <f>(Budget!J28)/2</f>
         <v>0</v>
       </c>
-      <c r="J13" s="67">
+      <c r="J13" s="36">
         <f>(Budget!L29)/2</f>
         <v>0</v>
       </c>
-      <c r="K13" s="68">
+      <c r="K13" s="40">
         <f>(Budget!L28)/2</f>
         <v>0</v>
       </c>
-      <c r="L13" s="67">
+      <c r="L13" s="36">
         <f>(Budget!N29)/2</f>
         <v>0</v>
       </c>
-      <c r="M13" s="68">
+      <c r="M13" s="40">
         <f>(Budget!N28)/2</f>
         <v>0</v>
       </c>
-      <c r="N13" s="70"/>
-      <c r="O13" s="70"/>
-      <c r="P13" s="70"/>
-      <c r="Q13" s="71"/>
-      <c r="R13" s="71"/>
-      <c r="S13" s="71"/>
-      <c r="T13" s="71"/>
-      <c r="U13" s="71"/>
-      <c r="V13" s="71"/>
-      <c r="W13" s="71"/>
+      <c r="N13" s="14"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="14"/>
+      <c r="Q13" s="15"/>
+      <c r="R13" s="15"/>
+      <c r="S13" s="15"/>
+      <c r="T13" s="15"/>
+      <c r="U13" s="15"/>
+      <c r="V13" s="15"/>
+      <c r="W13" s="15"/>
       <c r="X13" s="15"/>
       <c r="Y13" s="15"/>
       <c r="Z13" s="15"/>
       <c r="AA13" s="15"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="67">
+      <c r="B14" s="36">
         <f>(Budget!D32)/2</f>
         <v>0</v>
       </c>
-      <c r="C14" s="68">
+      <c r="C14" s="40">
         <f>(Budget!D31)/2</f>
         <v>0</v>
       </c>
-      <c r="D14" s="67">
+      <c r="D14" s="36">
         <f>(Budget!F32)/2</f>
         <v>0</v>
       </c>
-      <c r="E14" s="68">
+      <c r="E14" s="40">
         <f>(Budget!F31)/2</f>
         <v>0</v>
       </c>
-      <c r="F14" s="67">
+      <c r="F14" s="36">
         <f>(Budget!H32)/2</f>
         <v>0</v>
       </c>
-      <c r="G14" s="68">
+      <c r="G14" s="40">
         <f>(Budget!H31)/2</f>
         <v>0</v>
       </c>
-      <c r="H14" s="67">
+      <c r="H14" s="36">
         <f>(Budget!J32)/2</f>
         <v>0</v>
       </c>
-      <c r="I14" s="68">
+      <c r="I14" s="40">
         <f>(Budget!J31)/2</f>
         <v>0</v>
       </c>
-      <c r="J14" s="67">
+      <c r="J14" s="36">
         <f>(Budget!L32)/2</f>
         <v>0</v>
       </c>
-      <c r="K14" s="68">
+      <c r="K14" s="40">
         <f>(Budget!L31)/2</f>
         <v>0</v>
       </c>
-      <c r="L14" s="67">
+      <c r="L14" s="36">
         <f>(Budget!N32)/2</f>
         <v>0</v>
       </c>
-      <c r="M14" s="68">
+      <c r="M14" s="40">
         <f>(Budget!N31)/2</f>
         <v>0</v>
       </c>
-      <c r="N14" s="70"/>
-      <c r="O14" s="70"/>
-      <c r="P14" s="70"/>
-      <c r="Q14" s="71"/>
-      <c r="R14" s="71"/>
-      <c r="S14" s="71"/>
-      <c r="T14" s="71"/>
-      <c r="U14" s="71"/>
-      <c r="V14" s="71"/>
-      <c r="W14" s="71"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="14"/>
+      <c r="P14" s="14"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
+      <c r="T14" s="15"/>
+      <c r="U14" s="15"/>
+      <c r="V14" s="15"/>
+      <c r="W14" s="15"/>
       <c r="X14" s="15"/>
       <c r="Y14" s="15"/>
       <c r="Z14" s="15"/>
       <c r="AA14" s="15"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="67">
+      <c r="B15" s="36">
         <f>(Budget!D35)/2</f>
         <v>0</v>
       </c>
-      <c r="C15" s="68">
+      <c r="C15" s="40">
         <f>(Budget!D34)/2</f>
         <v>0</v>
       </c>
-      <c r="D15" s="67">
+      <c r="D15" s="36">
         <f>(Budget!F35)/2</f>
         <v>0</v>
       </c>
-      <c r="E15" s="68">
+      <c r="E15" s="40">
         <f>(Budget!F34)/2</f>
         <v>0</v>
       </c>
-      <c r="F15" s="67">
+      <c r="F15" s="36">
         <f>(Budget!H35)/2</f>
         <v>0</v>
       </c>
-      <c r="G15" s="68">
+      <c r="G15" s="40">
         <f>(Budget!H34)/2</f>
         <v>0</v>
       </c>
-      <c r="H15" s="67">
+      <c r="H15" s="36">
         <f>(Budget!J35)/2</f>
         <v>0</v>
       </c>
-      <c r="I15" s="68">
+      <c r="I15" s="40">
         <f>(Budget!J34)/2</f>
         <v>0</v>
       </c>
-      <c r="J15" s="67">
+      <c r="J15" s="36">
         <f>(Budget!L35)/2</f>
         <v>0</v>
       </c>
-      <c r="K15" s="68">
+      <c r="K15" s="40">
         <f>(Budget!L34)/2</f>
         <v>0</v>
       </c>
-      <c r="L15" s="67">
+      <c r="L15" s="36">
         <f>(Budget!N35)/2</f>
         <v>0</v>
       </c>
-      <c r="M15" s="68">
+      <c r="M15" s="40">
         <f>(Budget!N34)/2</f>
         <v>0</v>
       </c>
-      <c r="N15" s="70"/>
-      <c r="O15" s="70"/>
-      <c r="P15" s="70"/>
-      <c r="Q15" s="71"/>
-      <c r="R15" s="71"/>
-      <c r="S15" s="71"/>
-      <c r="T15" s="71"/>
-      <c r="U15" s="71"/>
-      <c r="V15" s="71"/>
-      <c r="W15" s="71"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="14"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="15"/>
+      <c r="S15" s="15"/>
+      <c r="T15" s="15"/>
+      <c r="U15" s="15"/>
+      <c r="V15" s="15"/>
+      <c r="W15" s="15"/>
       <c r="X15" s="15"/>
       <c r="Y15" s="15"/>
       <c r="Z15" s="15"/>
       <c r="AA15" s="15"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="67">
+      <c r="B16" s="36">
         <f>(Budget!D38)/2</f>
         <v>0</v>
       </c>
-      <c r="C16" s="68">
+      <c r="C16" s="40">
         <f>(Budget!D37)/2</f>
         <v>0</v>
       </c>
-      <c r="D16" s="67">
+      <c r="D16" s="36">
         <f>(Budget!F38)/2</f>
         <v>0</v>
       </c>
-      <c r="E16" s="68">
+      <c r="E16" s="40">
         <f>(Budget!F37)/2</f>
         <v>0</v>
       </c>
-      <c r="F16" s="67">
+      <c r="F16" s="36">
         <f>(Budget!H38)/2</f>
         <v>0</v>
       </c>
-      <c r="G16" s="68">
+      <c r="G16" s="40">
         <f>(Budget!H37)/2</f>
         <v>0</v>
       </c>
-      <c r="H16" s="67">
+      <c r="H16" s="36">
         <f>(Budget!J38)/2</f>
         <v>0</v>
       </c>
-      <c r="I16" s="68">
+      <c r="I16" s="40">
         <f>(Budget!J37)/2</f>
         <v>0</v>
       </c>
-      <c r="J16" s="67">
+      <c r="J16" s="36">
         <f>(Budget!L38)/2</f>
         <v>0</v>
       </c>
-      <c r="K16" s="68">
+      <c r="K16" s="40">
         <f>(Budget!L37)/2</f>
         <v>0</v>
       </c>
-      <c r="L16" s="67">
+      <c r="L16" s="36">
         <f>(Budget!N38)/2</f>
         <v>0</v>
       </c>
-      <c r="M16" s="68">
+      <c r="M16" s="40">
         <f>(Budget!N37)/2</f>
         <v>0</v>
       </c>
-      <c r="N16" s="70"/>
-      <c r="O16" s="70"/>
-      <c r="P16" s="70"/>
-      <c r="Q16" s="71"/>
-      <c r="R16" s="71"/>
-      <c r="S16" s="71"/>
-      <c r="T16" s="71"/>
-      <c r="U16" s="71"/>
-      <c r="V16" s="71"/>
-      <c r="W16" s="71"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+      <c r="V16" s="15"/>
+      <c r="W16" s="15"/>
       <c r="X16" s="15"/>
       <c r="Y16" s="15"/>
       <c r="Z16" s="15"/>
@@ -31860,130 +31864,130 @@
       <c r="A17" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="67">
+      <c r="B17" s="36">
         <f>(Budget!D39)/2</f>
         <v>0</v>
       </c>
-      <c r="C17" s="68">
+      <c r="C17" s="40">
         <f>B17</f>
         <v>0</v>
       </c>
-      <c r="D17" s="67"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="67"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="67"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="67"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="67"/>
-      <c r="M17" s="68"/>
-      <c r="N17" s="71"/>
-      <c r="O17" s="71"/>
-      <c r="P17" s="71"/>
-      <c r="Q17" s="71"/>
-      <c r="R17" s="71"/>
-      <c r="S17" s="71"/>
-      <c r="T17" s="71"/>
-      <c r="U17" s="71"/>
-      <c r="V17" s="71"/>
-      <c r="W17" s="71"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="36"/>
+      <c r="K17" s="40"/>
+      <c r="L17" s="36"/>
+      <c r="M17" s="40"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="15"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+      <c r="V17" s="15"/>
+      <c r="W17" s="15"/>
       <c r="X17" s="15"/>
       <c r="Y17" s="15"/>
       <c r="Z17" s="15"/>
       <c r="AA17" s="15"/>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="72">
+      <c r="B18" s="30">
         <f t="shared" ref="B18:M18" si="0">SUM(B4:B17)</f>
         <v>0</v>
       </c>
-      <c r="C18" s="73">
+      <c r="C18" s="51">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D18" s="72">
+      <c r="D18" s="30">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E18" s="73">
+      <c r="E18" s="51">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F18" s="72">
+      <c r="F18" s="30">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G18" s="73">
+      <c r="G18" s="51">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="72">
+      <c r="H18" s="30">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I18" s="73">
+      <c r="I18" s="51">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="72">
+      <c r="J18" s="30">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K18" s="73">
+      <c r="K18" s="51">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L18" s="72">
+      <c r="L18" s="30">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M18" s="73">
+      <c r="M18" s="51">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N18" s="70"/>
-      <c r="O18" s="70"/>
-      <c r="P18" s="71"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="70"/>
-      <c r="S18" s="70"/>
-      <c r="T18" s="70"/>
-      <c r="U18" s="70"/>
-      <c r="V18" s="70"/>
-      <c r="W18" s="70"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="14"/>
+      <c r="U18" s="14"/>
+      <c r="V18" s="14"/>
+      <c r="W18" s="14"/>
       <c r="X18" s="14"/>
       <c r="Y18" s="14"/>
       <c r="Z18" s="14"/>
       <c r="AA18" s="14"/>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A19" s="36"/>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="54"/>
-      <c r="D19" s="54"/>
-      <c r="E19" s="61">
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="63">
         <f>E1-SUM(B18+D18+F18+H18+J18+L18)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="54"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="60" t="s">
+      <c r="F19" s="58"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="I19" s="54"/>
-      <c r="J19" s="54"/>
-      <c r="K19" s="61">
+      <c r="I19" s="58"/>
+      <c r="J19" s="58"/>
+      <c r="K19" s="63">
         <f>K1-SUM(C18+E18+G18+I18+K18+M18)</f>
         <v>0</v>
       </c>
-      <c r="L19" s="54"/>
-      <c r="M19" s="58"/>
+      <c r="L19" s="58"/>
+      <c r="M19" s="62"/>
       <c r="N19" s="15"/>
       <c r="O19" s="15"/>
       <c r="P19" s="15"/>
@@ -31999,7 +32003,7 @@
       <c r="Z19" s="15"/>
       <c r="AA19" s="15"/>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A20" s="36"/>
       <c r="B20" s="36"/>
       <c r="C20" s="40"/>
@@ -32028,7 +32032,7 @@
       <c r="Z20" s="15"/>
       <c r="AA20" s="15"/>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A21" s="36"/>
       <c r="B21" s="36"/>
       <c r="C21" s="40"/>
@@ -32057,7 +32061,7 @@
       <c r="Z21" s="15"/>
       <c r="AA21" s="15"/>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A22" s="36"/>
       <c r="B22" s="36"/>
       <c r="C22" s="40"/>
@@ -32086,7 +32090,7 @@
       <c r="Z22" s="15"/>
       <c r="AA22" s="15"/>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A23" s="36"/>
       <c r="B23" s="36"/>
       <c r="C23" s="40"/>
@@ -32115,7 +32119,7 @@
       <c r="Z23" s="15"/>
       <c r="AA23" s="15"/>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A24" s="36"/>
       <c r="B24" s="36"/>
       <c r="C24" s="40"/>
@@ -32144,7 +32148,7 @@
       <c r="Z24" s="15"/>
       <c r="AA24" s="15"/>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A25" s="36"/>
       <c r="B25" s="36"/>
       <c r="C25" s="40"/>
@@ -32173,7 +32177,7 @@
       <c r="Z25" s="15"/>
       <c r="AA25" s="15"/>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A26" s="36"/>
       <c r="B26" s="36"/>
       <c r="C26" s="40"/>
@@ -32202,7 +32206,7 @@
       <c r="Z26" s="15"/>
       <c r="AA26" s="15"/>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="36"/>
       <c r="B27" s="36"/>
       <c r="C27" s="40"/>
@@ -32231,7 +32235,7 @@
       <c r="Z27" s="15"/>
       <c r="AA27" s="15"/>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A28" s="36"/>
       <c r="B28" s="36"/>
       <c r="C28" s="40"/>
@@ -32260,7 +32264,7 @@
       <c r="Z28" s="15"/>
       <c r="AA28" s="15"/>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A29" s="36"/>
       <c r="B29" s="36"/>
       <c r="C29" s="40"/>
@@ -32289,7 +32293,7 @@
       <c r="Z29" s="15"/>
       <c r="AA29" s="15"/>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A30" s="36"/>
       <c r="B30" s="36"/>
       <c r="C30" s="40"/>
@@ -59754,6 +59758,52 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{868CC755-70DE-4065-A09A-50FAB03E917E}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.5546875" customWidth="1"/>
+    <col min="2" max="3" width="17.88671875" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" style="54" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="64" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="52" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="53" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="54">
+        <f>B3/2</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -59765,10 +59815,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="70" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="58"/>
       <c r="C1" s="42"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>